<commit_message>
feat: organize rogue card artwork through the Excel production pipeline
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeRogueCards.xlsx
+++ b/data/Excel/GuLiStrikeRogueCards.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>id</t>
   </si>
@@ -324,6 +324,12 @@
   </si>
   <si>
     <t>己方本局当前及后续重防号：雨点攻势。完整齐射数量每次加1，基础1发，每队本局最多59次，单台上限60发。</t>
+  </si>
+  <si>
+    <t>ArtworkId</t>
+  </si>
+  <si>
+    <t>整数，引用GuLiStrikeCardArtwork.xlsx/Artworks.id；导出为既有FrontMaterial，不在源表重复维护材质路径。</t>
   </si>
 </sst>
 </file>
@@ -714,7 +720,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>61</v>
@@ -764,7 +770,7 @@
         <v>13</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J2" t="s">
         <v>14</v>
@@ -863,8 +869,8 @@
       <c r="H4">
         <v>0.2</v>
       </c>
-      <c r="I4" t="s">
-        <v>56</v>
+      <c r="I4">
+        <v>1</v>
       </c>
       <c r="J4" t="s">
         <v>62</v>
@@ -913,8 +919,8 @@
       <c r="H5">
         <v>0.5</v>
       </c>
-      <c r="I5" t="s">
-        <v>57</v>
+      <c r="I5">
+        <v>2</v>
       </c>
       <c r="J5" t="s">
         <v>62</v>
@@ -963,8 +969,8 @@
       <c r="H6">
         <v>0.2</v>
       </c>
-      <c r="I6" t="s">
-        <v>58</v>
+      <c r="I6">
+        <v>3</v>
       </c>
       <c r="J6" t="s">
         <v>62</v>
@@ -1013,8 +1019,8 @@
       <c r="H7">
         <v>0</v>
       </c>
-      <c r="I7" t="s">
-        <v>95</v>
+      <c r="I7">
+        <v>4</v>
       </c>
       <c r="J7" t="s">
         <v>62</v>
@@ -1063,8 +1069,8 @@
       <c r="H8">
         <v>0</v>
       </c>
-      <c r="I8" t="s">
-        <v>101</v>
+      <c r="I8">
+        <v>5</v>
       </c>
       <c r="J8" t="s">
         <v>62</v>
@@ -1174,10 +1180,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11">

</xml_diff>